<commit_message>
Merge US01 into fisheries department
</commit_message>
<xml_diff>
--- a/data/11508/系所經費代碼與中文名稱對照表.xlsx
+++ b/data/11508/系所經費代碼與中文名稱對照表.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\IR大數據分析組\IR-躍升相關\經費收支明細\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\projects\BudgetDashboard\data\11508\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19E43302-C45D-4D91-B716-8129F875AEB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6D50B6A-8AF3-4991-8AE3-DF4C7E56F6D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A410AB86-5814-4FCF-ADFA-7EA48B0B568D}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="118">
   <si>
     <r>
       <rPr>
@@ -1106,6 +1106,10 @@
   </si>
   <si>
     <t>UT02</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>US01</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -1113,7 +1117,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1168,6 +1172,12 @@
       <family val="4"/>
       <charset val="136"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -1371,7 +1381,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1427,6 +1437,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1743,7 +1756,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D452D504-C59B-4FEE-9796-EA0E20A0674F}">
-  <dimension ref="A1:D55"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.125" bestFit="1" customWidth="1"/>
@@ -2234,11 +2247,11 @@
       <c r="A44" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B44" s="12" t="s">
-        <v>111</v>
-      </c>
-      <c r="C44" s="11" t="s">
-        <v>110</v>
+      <c r="B44" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="C44" s="19" t="s">
+        <v>117</v>
       </c>
       <c r="D44" t="s">
         <v>109</v>
@@ -2246,46 +2259,49 @@
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="B45" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="C45" s="6" t="s">
-        <v>85</v>
+        <v>17</v>
+      </c>
+      <c r="B45" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="C45" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="D45" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>42</v>
+        <v>83</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="4" t="s">
-        <v>17</v>
+        <v>42</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>83</v>
+        <v>17</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -2293,21 +2309,21 @@
         <v>83</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
@@ -2315,10 +2331,10 @@
         <v>94</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
@@ -2326,42 +2342,53 @@
         <v>94</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="4" t="s">
-        <v>6</v>
+        <v>94</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B54" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B54" s="5" t="s">
+      <c r="B55" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="C54" s="6" t="s">
+      <c r="C55" s="6" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="55" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="8" t="s">
+    <row r="56" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B55" s="9" t="s">
+      <c r="B56" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="C55" s="10" t="s">
+      <c r="C56" s="10" t="s">
         <v>106</v>
       </c>
     </row>

</xml_diff>